<commit_message>
Ajout Valence, Chambéry, Avignon, Cannes/Antibes + décisionnaires Pappers
Tableau consolidé (8 villes, 153 agences/agents) avec numéros mobiles 06/07.
Noms des décisionnaires enrichis via Pappers (gérant/président) quand
disponibles. Exclusions: chasseurs, conciergeries, viagers, gestions
locatives pures, conseillers en gestion de patrimoine.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyLHb8pJT5tJXvWVQCChTK
</commit_message>
<xml_diff>
--- a/agences_immobilieres_06_07.xlsx
+++ b/agences_immobilieres_06_07.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Agences immobilières" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agences immobilières'!$A$1:$D$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agences immobilières'!$A$1:$D$154</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,12 +459,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -2056,8 +2056,1588 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Ambiance Immobilier</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Mireille Mugler-Filliat</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>06 60 71 10 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Stéphanie Garcia - Conseiller Immobilier IAD</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Stéphanie Garcia</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>06 41 96 28 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Agence immobilière Korine Olivier</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Korine Olivier</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>06 69 28 43 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>3%.Com Valence (3ComImmo)</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>06 30 52 41 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>La Carte immobilière !</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Alexandre Dalla Costa</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>07 83 39 17 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>L'Immo</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr"/>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>06 75 67 44 87</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>L et N Immobilier</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr"/>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>06 14 20 14 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Tanguy Marlhens Immobilier IAD</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Tanguy Marlhens</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>06 45 78 42 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Sandra Dubois - IKAMI</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Sandra Dubois</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>06 45 29 33 64</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Veronique Blanc Immobilier</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Véronique Blanc</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>06 71 10 19 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Agence Kévork'Immobilier</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Sylvie Maldjian</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>06 20 60 05 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Hapiness Immo</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr"/>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>07 61 92 72 06</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Philippe Champagne - Cimm Immobilier</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Philippe Champagne</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>06 27 85 67 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Ids Immobilier</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr"/>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>06 08 84 78 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>3Link Immobilier Valence</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr"/>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>06 20 79 71 96</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Guillaume Rocheblave - 3G Immobilier</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Guillaume Rocheblave</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>06 99 88 73 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>Valence</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Groupe Clef d'Or Immobilier</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Florent Breton</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>06 23 74 96 90</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>ISI Immobilier Savoie Investissement</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Laurent Leoni</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>06 09 45 05 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Mathurin Immobilier</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr"/>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>07 83 96 01 92</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>AS Immobilier</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr"/>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>07 65 15 87 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Muriel Terrié - Safti Immobilier</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>Muriel Terrié</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>06 70 48 14 05</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Loft'n co Immobilier</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr"/>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>06 81 08 31 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>AXO Immobilier</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr"/>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>06 61 84 04 61</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Trèfle Immobilier</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Sébastien &amp; Carine Rastel</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>06 17 61 04 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>EMC-Immo</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>Eric Monmaille</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>06 67 44 01 39</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Cabinet Valmer</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr"/>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>06 27 06 01 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>EffiCity - Romain Estivalet</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>Romain Estivalet</t>
+        </is>
+      </c>
+      <c r="D105" s="5" t="inlineStr">
+        <is>
+          <t>06 24 64 28 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Thomas Audy - Capifrance</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Thomas Audy</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>06 11 49 51 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>Audrey Valaud - SAFTI</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>Audrey Valaud</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>06 69 22 61 63</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Javier Donoso Moretti - BSK Immobilier</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Javier Donoso Moretti</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>06 75 04 95 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Immobilier Excoffon Pascale</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Pascale Excoffon</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
+        <is>
+          <t>06 70 48 94 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Neovy Consulting</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Dylan Vie</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>06 83 33 38 53</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Yvan Duchemann</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>Yvan Duchemann</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
+        <is>
+          <t>06 43 83 68 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Sylvie Guicherd - Immobilier professionnel</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Sylvie Guicherd</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>06 79 27 04 91</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>Chambéry</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Nicolas Donjon - Comparet Immobilier</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>Nicolas Donjon</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>06 87 26 41 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Act'immo Avignon</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Benjamin Caillot</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>06 68 40 38 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Cynthia Dal Bello - Immobilier</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>Cynthia Dal Bello</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
+        <is>
+          <t>06 62 69 14 05</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>N&amp;F Immobilier</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Nicolas &amp; Félicie</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>06 98 28 16 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>LBH Immobilier</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>Hélène &amp; Barbara Bassard</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>06 51 62 83 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Laurent Bonnet - SAFTI</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Laurent Bonnet</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>06 09 69 01 61</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Rohart Immobilier</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Vincent Rohart</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>06 08 01 07 99</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Jérôme Durand Immobilier</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Jérôme Durand</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>06 70 87 47 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>De Bazelaire Immobilier</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Jean-Guy de Bazelaire</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
+        <is>
+          <t>06 74 36 24 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Aicha Lajournade - SAFTI</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Aicha Lajournade</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>06 25 68 48 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Prestig'Immo Office</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>Josette Blanc</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>06 11 45 63 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>123webimmo Avignon</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr"/>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>06 95 25 58 88</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>Agence Hérys Immo</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>Stéphanie Perdriolle (Pichot)</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>06 51 55 42 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>La Muse Immobilière</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr"/>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>06 12 24 89 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>Grégory Maulet</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>Grégory Maulet</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>07 69 37 09 98</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Naomi Hirst - SAFTI</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Naomi Hirst</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>07 70 28 28 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t>Matthias Ringenbach - SAFTI</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>Matthias Ringenbach</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>06 99 40 62 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Propriétés-Privées.com Avignon</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr"/>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>06 72 99 95 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>Talbot Propriétés</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>Geneviève Talbot (Klieber)</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>06 16 49 59 06</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Avignon</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Clicvente</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr"/>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>06 59 87 91 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>IMOP Cannes</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr"/>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>06 03 31 38 98</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Agence Alexander Claus</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Claus</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>06 03 83 39 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>Agence 57</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>Xavier Gruat</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>06 11 89 84 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Riva Immobilier</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Paolo Daelli</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>06 67 90 80 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>Limandat Real Estate</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>Chrystèle Limandat</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>06 63 64 86 56</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>123Webimmo Antibes</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr"/>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>06 03 17 27 88</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Jérôme Magnoli - Infinity Group Immobilier</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>Jérôme Magnoli</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>06 36 47 89 39</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>SP Real Estate Croisette</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr"/>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>06 03 62 11 03</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>Darkstone Estate Agency</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr"/>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>07 80 91 87 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Jan Valentin Darmstadt - JVD Immobilier</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Jan Valentin Darmstadt</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>07 86 03 55 05</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>Cyril Dubois - Expertimo</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>Cyril Dubois</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>06 50 67 13 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Agence JAMA Immobilier</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Marc Henry</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>06 14 99 90 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Phygital.immo</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>Sébastien Vidal</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>06 58 47 17 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Efficity (Stéphanie Fauré)</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Stéphanie Fauré</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>06 62 89 00 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>La Vida Riviera Immobilier</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr"/>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>06 23 68 22 91</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Palm Immo</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr"/>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>06 52 16 45 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>Providence Properties</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr"/>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>06 13 05 03 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Gwen Leroux - Conseillère Immobilier</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Gwen Leroux</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>06 17 97 72 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Expertimo Antibes - JF Guittard</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>Jean-François Guittard</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>06 09 68 47 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Adrien Rallo - Agent Immobilier</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Adrien Rallo</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>07 86 90 97 55</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>CD Immobilier Cannes</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="inlineStr"/>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>06 22 79 12 56</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Cannes / Antibes</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Zanchi - BSK Immobilier</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Alexandra Zanchi</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>06 21 11 46 74</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D78"/>
+  <autoFilter ref="A1:D154"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>